<commit_message>
Add Doubao TTS provider and refreshed job feed
</commit_message>
<xml_diff>
--- a/archive/2026-06-17/job.xlsx
+++ b/archive/2026-06-17/job.xlsx
@@ -2917,7 +2917,7 @@
       </c>
       <c r="V8" s="48" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；非招聘软件或页面未公开HR活跃状态</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；非招聘软件或页面未公开HR活跃状态</t>
         </is>
       </c>
       <c r="W8" s="48" t="inlineStr">
@@ -3436,7 +3436,7 @@
       </c>
       <c r="V11" s="48" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
+          <t>2026-06-17 自动复核：链接无法精确确认（403），需二次确认；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
         </is>
       </c>
       <c r="W11" s="48" t="inlineStr">
@@ -3482,17 +3482,17 @@
       </c>
       <c r="AF11" s="2" t="inlineStr">
         <is>
-          <t>A档，100分；字段显示主线为主线B-AI应用落地/AI产品工程师，匹配度高，原申请优先级P1主攻。城市/薪资为香港、HK$22,000-28,000/月，薪资匹配为部分达标，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：香港本地Agentic AI平台公司，主打企业客服与销售流程自动化；JD与可信度为中高、中高，入池岗位。关键风险：英文/粤语/IANG。</t>
+          <t>A档，100分；字段显示主线为主线B-AI应用落地/AI产品工程师，匹配度高，原申请优先级P1主攻。城市/薪资为香港、HK$22,000-28,000/月，薪资匹配为部分达标，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：香港本地Agentic AI平台公司，主打企业客服与销售流程自动化；JD与可信度为中高、中高，入池岗位。关键风险：英文/粤语/IANG；招聘状态不稳。</t>
         </is>
       </c>
       <c r="AG11" s="2" t="inlineStr">
         <is>
-          <t>重点准备后投</t>
+          <t>先核验再投</t>
         </is>
       </c>
       <c r="AH11" s="2" t="inlineStr">
         <is>
-          <t>英文/粤语/IANG</t>
+          <t>英文/粤语/IANG；招聘状态不稳</t>
         </is>
       </c>
       <c r="AI11" s="2" t="inlineStr">
@@ -4820,7 +4820,7 @@
       </c>
       <c r="V19" s="48" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；非招聘软件或页面未公开HR活跃状态</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；非招聘软件或页面未公开HR活跃状态</t>
         </is>
       </c>
       <c r="W19" s="48" t="inlineStr">
@@ -4993,7 +4993,7 @@
       </c>
       <c r="V20" s="48" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；非招聘软件或页面未公开HR活跃状态</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；非招聘软件或页面未公开HR活跃状态</t>
         </is>
       </c>
       <c r="W20" s="48" t="inlineStr">
@@ -5339,7 +5339,7 @@
       </c>
       <c r="V22" s="48" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；非招聘软件或页面未公开HR活跃状态</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；非招聘软件或页面未公开HR活跃状态</t>
         </is>
       </c>
       <c r="W22" s="48" t="inlineStr">
@@ -7519,7 +7519,7 @@
       </c>
       <c r="V12" s="47" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
         </is>
       </c>
       <c r="W12" s="47" t="inlineStr">
@@ -7865,7 +7865,7 @@
       </c>
       <c r="V14" s="47" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
         </is>
       </c>
       <c r="W14" s="47" t="inlineStr">
@@ -8384,7 +8384,7 @@
       </c>
       <c r="V17" s="48" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
         </is>
       </c>
       <c r="W17" s="48" t="inlineStr">
@@ -8557,7 +8557,7 @@
       </c>
       <c r="V18" s="48" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接无法精确确认（429），需二次确认；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
         </is>
       </c>
       <c r="W18" s="48" t="inlineStr">
@@ -8599,21 +8599,21 @@
         </is>
       </c>
       <c r="AE18" s="2" t="n">
-        <v>87</v>
+        <v>98</v>
       </c>
       <c r="AF18" s="2" t="inlineStr">
         <is>
-          <t>A档，87分；字段显示主线为备线C-AI解决方案/数字化产品，匹配度中高，原申请优先级P3练手/备选实习。城市/薪资为深圳、未写，薪资匹配为实习可接受，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：腾讯云CSIG，中国头部云与产业互联网平台，做云、AI、安全和行业数字化；JD与可信度为精确JD、高，入池岗位。关键风险：出差/驻厂；招聘状态不稳。</t>
+          <t>A档，98分；字段显示主线为备线C-AI解决方案/数字化产品，匹配度中高，原申请优先级P3练手/备选实习。城市/薪资为深圳、未写，薪资匹配为实习可接受，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：腾讯云CSIG，中国头部云与产业互联网平台，做云、AI、安全和行业数字化；JD与可信度为精确JD、高，入池岗位。关键风险：出差/驻厂。</t>
         </is>
       </c>
       <c r="AG18" s="2" t="inlineStr">
         <is>
-          <t>先核验再投</t>
+          <t>定制简历后优先投</t>
         </is>
       </c>
       <c r="AH18" s="2" t="inlineStr">
         <is>
-          <t>出差/驻厂；招聘状态不稳</t>
+          <t>出差/驻厂</t>
         </is>
       </c>
       <c r="AI18" s="2" t="inlineStr">
@@ -9941,7 +9941,7 @@
       </c>
       <c r="V26" s="48" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；非招聘软件或页面未公开HR活跃状态</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；非招聘软件或页面未公开HR活跃状态</t>
         </is>
       </c>
       <c r="W26" s="48" t="inlineStr">
@@ -10460,7 +10460,7 @@
       </c>
       <c r="V29" s="47" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接无法精确确认（429），需二次确认；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
         </is>
       </c>
       <c r="W29" s="47" t="inlineStr">
@@ -10506,7 +10506,7 @@
       </c>
       <c r="AF29" s="2" t="inlineStr">
         <is>
-          <t>B档，79分；字段显示主线为主线A-AIoT/AI终端/软硬件产品，匹配度高，原申请优先级P1主线实习。城市/薪资为深圳、400-500/天待确认，薪资匹配为实习可接受，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：深圳创客硬件和桌面激光加工设备出海品牌，软硬件结合和创作者生态强；JD与可信度为入口页/搜索页、中高，入池岗位。关键风险：薪资待确认；JD不精确；出差/驻厂；招聘状态不稳。</t>
+          <t>B档，79分；字段显示主线为主线A-AIoT/AI终端/软硬件产品，匹配度高，原申请优先级P1主线实习。城市/薪资为深圳、400-500/天待确认，薪资匹配为实习可接受，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：深圳创客硬件和桌面激光加工设备出海品牌，软硬件结合和创作者生态强；JD与可信度为入口页/搜索页、中高，入池岗位。关键风险：薪资待确认；JD不精确；出差/驻厂。</t>
         </is>
       </c>
       <c r="AG29" s="2" t="inlineStr">
@@ -10516,7 +10516,7 @@
       </c>
       <c r="AH29" s="2" t="inlineStr">
         <is>
-          <t>薪资待确认；JD不精确；出差/驻厂；招聘状态不稳</t>
+          <t>薪资待确认；JD不精确；出差/驻厂</t>
         </is>
       </c>
       <c r="AI29" s="2" t="inlineStr">
@@ -11152,7 +11152,7 @@
       </c>
       <c r="V33" s="48" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接无法精确确认（429），需二次确认；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
         </is>
       </c>
       <c r="W33" s="48" t="inlineStr">
@@ -11194,11 +11194,11 @@
         </is>
       </c>
       <c r="AE33" s="2" t="n">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="AF33" s="2" t="inlineStr">
         <is>
-          <t>B档，69分；字段显示主线为主线B-AI应用落地/AI产品工程师，匹配度中高，原申请优先级P2AI应用实习。城市/薪资为香港/深圳、未公开，薪资匹配为实习可接受，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：移动设备管理、远程控制和跨设备协同工具公司，香港/深圳协同；JD与可信度为入口页/搜索页、中高，入池岗位。关键风险：薪资待确认；JD不精确；英文/粤语/IANG；出差/驻厂；招聘状态不稳。</t>
+          <t>B档，73分；字段显示主线为主线B-AI应用落地/AI产品工程师，匹配度中高，原申请优先级P2AI应用实习。城市/薪资为香港/深圳、未公开，薪资匹配为实习可接受，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：移动设备管理、远程控制和跨设备协同工具公司，香港/深圳协同；JD与可信度为入口页/搜索页、中高，入池岗位。关键风险：薪资待确认；JD不精确；英文/粤语/IANG；出差/驻厂。</t>
         </is>
       </c>
       <c r="AG33" s="2" t="inlineStr">
@@ -11208,7 +11208,7 @@
       </c>
       <c r="AH33" s="2" t="inlineStr">
         <is>
-          <t>薪资待确认；JD不精确；英文/粤语/IANG；出差/驻厂；招聘状态不稳</t>
+          <t>薪资待确认；JD不精确；英文/粤语/IANG；出差/驻厂</t>
         </is>
       </c>
       <c r="AI33" s="2" t="inlineStr">
@@ -11671,7 +11671,7 @@
       </c>
       <c r="V36" s="47" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；非招聘软件或页面未公开HR活跃状态</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；非招聘软件或页面未公开HR活跃状态</t>
         </is>
       </c>
       <c r="W36" s="47" t="inlineStr">
@@ -13750,7 +13750,7 @@
           <t>高</t>
         </is>
       </c>
-      <c r="AA48" s="17" t="inlineStr">
+      <c r="AA48" s="62" t="inlineStr">
         <is>
           <t>https://jobs.apple.com/en-us/details/200494847-3435/engineering-project-manager-intern-shanghai-shenzhen?team=HRDWR</t>
         </is>
@@ -13760,10 +13760,10 @@
       </c>
       <c r="AC48" s="47" t="inlineStr">
         <is>
-          <t>2026-06-17 Apple miss correction: official Jobs link grade fixed; promoted from expanded to internship.</t>
-        </is>
-      </c>
-      <c r="AD48" s="60" t="inlineStr">
+          <t>2026-06-17 Apple miss correction: official Jobs link grade fixed; promoted from expanded to internship.；首次入库日期=2026-06-17</t>
+        </is>
+      </c>
+      <c r="AD48" s="59" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -13773,12 +13773,12 @@
       </c>
       <c r="AF48" s="47" t="inlineStr">
         <is>
-          <t>B档，79分；字段显示主线为主线A-AI终端/智能硬件/TPM/软硬件协同项目，匹配度高，原申请优先级P2今日可投。城市/薪资为深圳/上海、Apple官网未公开，薪资匹配为实习薪资未公开；Apple平台价值高，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：全球消费电子与软硬件一体化顶级外企，AI终端、硬件工程、供应链和产品体验平台价值极高；JD与可信度为Apple官方搜索页可核验标题、发…、中高，扩源入口需后置核验。关键风险：薪资待确认；JD不精确；英文/粤语/IANG；招聘状态不稳。</t>
+          <t>B档，79分；字段显示主线为主线A-AI终端/智能硬件/TPM/软硬件协同项目，匹配度高，原申请优先级P2今日可投。城市/薪资为深圳/上海、Apple官网未公开，薪资匹配为实习薪资未公开；Apple平台价值高，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：全球消费电子与软硬件一体化顶级外企，AI终端、硬件工程、供应链和产品体验平台价值极高；JD与可信度为Apple官方搜索页可核验标题、发…、高，入池岗位。关键风险：薪资待确认；JD不精确；英文/粤语/IANG；招聘状态不稳。</t>
         </is>
       </c>
       <c r="AG48" s="47" t="inlineStr">
         <is>
-          <t>作为主投池，持续监控</t>
+          <t>二次核验后投</t>
         </is>
       </c>
       <c r="AH48" s="47" t="inlineStr">
@@ -14065,326 +14065,326 @@
       </c>
     </row>
     <row r="2" ht="56" customHeight="1">
-      <c r="A2" s="64" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B2" s="64" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>实习岗</t>
         </is>
       </c>
-      <c r="C2" s="64" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Apple</t>
         </is>
       </c>
-      <c r="D2" s="64" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Engineering Project Manager Intern-Shanghai/ Shenzhen</t>
         </is>
       </c>
-      <c r="E2" s="64" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>深圳/上海</t>
         </is>
       </c>
-      <c r="F2" s="64" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Apple官网未公开</t>
         </is>
       </c>
-      <c r="G2" s="64" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="H2" s="64" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>实习薪资未公开；Apple平台价值高</t>
         </is>
       </c>
-      <c r="I2" s="64" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>主线A-AI终端/智能硬件/TPM/软硬件协同项目</t>
         </is>
       </c>
-      <c r="J2" s="64" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>P2今日可投</t>
         </is>
       </c>
-      <c r="K2" s="64" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>中高</t>
         </is>
       </c>
-      <c r="L2" s="64" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>实习/硬件项目管理/EPM/外企</t>
         </is>
       </c>
-      <c r="M2" s="64" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>学生岗位，具体年级与专业以Apple JD为准</t>
         </is>
       </c>
-      <c r="N2" s="64" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Apple官网显示Intern岗位；完整JD为JS页面，需投前二次确认每周到岗、实习周期和技术要求</t>
         </is>
       </c>
-      <c r="O2" s="64" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>2026-06-11发布；2026-06-17官方搜索页可见</t>
         </is>
       </c>
-      <c r="P2" s="64" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>Apple Jobs</t>
         </is>
       </c>
-      <c r="Q2" s="64" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>全球消费电子与软硬件一体化顶级外企，AI终端、硬件工程、供应链和产品体验平台价值极高</t>
         </is>
       </c>
-      <c r="R2" s="64" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>硬件工程项目管理实习，预计围绕跨职能协作、项目节奏、工程问题跟进、样机/量产节点沟通和供应链协同。</t>
         </is>
       </c>
-      <c r="S2" s="64" t="inlineStr">
+      <c r="S2" t="inlineStr">
         <is>
           <t>外企英文沟通与硬件工程语境；可能偏EPM/执行协同而非产品定义；完整JD需二次确认。</t>
         </is>
       </c>
-      <c r="T2" s="64" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>英文风险中；代码风险低；算法风险低；驻厂/供应链沟通风险中。</t>
         </is>
       </c>
-      <c r="U2" s="64" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>Apple官方搜索页可核验标题、发布时间、地点和Role Number；详情页JS渲染，职责需二次确认</t>
         </is>
       </c>
-      <c r="V2" s="64" t="inlineStr">
+      <c r="V2" t="inlineStr">
         <is>
           <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；非招聘软件或页面未公开HR活跃状态</t>
         </is>
       </c>
-      <c r="W2" s="64" t="inlineStr">
+      <c r="W2" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="X2" s="64" t="inlineStr">
+      <c r="X2" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="Y2" s="64" t="inlineStr">
+      <c r="Y2" t="inlineStr">
         <is>
           <t>Apple智能硬件/TPM版：突出工业设计、硬件产品、CMF、AI硕士、跨团队项目协作、英文沟通和软硬件结合项目。</t>
         </is>
       </c>
-      <c r="Z2" s="64" t="inlineStr">
+      <c r="Z2" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="AA2" s="17" t="inlineStr">
+      <c r="AA2" s="50" t="inlineStr">
         <is>
           <t>https://jobs.apple.com/en-us/details/200494847-3435/engineering-project-manager-intern-shanghai-shenzhen?team=HRDWR</t>
         </is>
       </c>
-      <c r="AB2" s="64" t="inlineStr">
+      <c r="AB2" s="53" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="AC2" s="64" t="n">
+      <c r="AC2" s="2" t="n">
         <v>79</v>
       </c>
-      <c r="AD2" s="64" t="inlineStr">
-        <is>
-          <t>B档，79分；字段显示主线为主线A-AI终端/智能硬件/TPM/软硬件协同项目，匹配度高，原申请优先级P2今日可投。城市/薪资为深圳/上海、Apple官网未公开，薪资匹配为实习薪资未公开；Apple平台价值高，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：全球消费电子与软硬件一体化顶级外企，AI终端、硬件工程、供应链和产品体验平台价值极高；JD与可信度为Apple官方搜索页可核验标题、发…、中高，扩源入口需后置核验。关键风险：薪资待确认；JD不精确；英文/粤语/IANG；招聘状态不稳。</t>
-        </is>
-      </c>
-      <c r="AE2" s="64" t="inlineStr">
-        <is>
-          <t>作为主投池，持续监控</t>
-        </is>
-      </c>
-      <c r="AF2" s="64" t="inlineStr">
+      <c r="AD2" s="2" t="inlineStr">
+        <is>
+          <t>B档，79分；字段显示主线为主线A-AI终端/智能硬件/TPM/软硬件协同项目，匹配度高，原申请优先级P2今日可投。城市/薪资为深圳/上海、Apple官网未公开，薪资匹配为实习薪资未公开；Apple平台价值高，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：全球消费电子与软硬件一体化顶级外企，AI终端、硬件工程、供应链和产品体验平台价值极高；JD与可信度为Apple官方搜索页可核验标题、发…、高，入池岗位。关键风险：薪资待确认；JD不精确；英文/粤语/IANG；招聘状态不稳。</t>
+        </is>
+      </c>
+      <c r="AE2" s="2" t="inlineStr">
+        <is>
+          <t>二次核验后投</t>
+        </is>
+      </c>
+      <c r="AF2" s="2" t="inlineStr">
         <is>
           <t>薪资待确认；JD不精确；英文/粤语/IANG；招聘状态不稳</t>
         </is>
       </c>
-      <c r="AG2" s="64" t="inlineStr">
+      <c r="AG2" s="2" t="inlineStr">
         <is>
           <t>Apple智能硬件/TPM版：突出工业设计、硬件产品、CMF、AI硕士、跨团队项目协作、英文沟通和软硬件结合项目。</t>
         </is>
       </c>
     </row>
     <row r="3" ht="56" customHeight="1">
-      <c r="A3" s="64" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="B3" s="64" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>次选_条件不完全符合</t>
         </is>
       </c>
-      <c r="C3" s="64" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Apple</t>
         </is>
       </c>
-      <c r="D3" s="64" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Technical Program Manager, iPad</t>
         </is>
       </c>
-      <c r="E3" s="64" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>深圳</t>
         </is>
       </c>
-      <c r="F3" s="64" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Apple官网未公开</t>
         </is>
       </c>
-      <c r="G3" s="64" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>中高</t>
         </is>
       </c>
-      <c r="H3" s="64" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>薪资未知；Apple平台价值高</t>
         </is>
       </c>
-      <c r="I3" s="64" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>主线A-AI终端/智能硬件/TPM/NPI</t>
         </is>
       </c>
-      <c r="J3" s="64" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>P3二次确认后投递</t>
         </is>
       </c>
-      <c r="K3" s="64" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>中高</t>
         </is>
       </c>
-      <c r="L3" s="64" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>正式/TPM/智能硬件/外企</t>
         </is>
       </c>
-      <c r="M3" s="64" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>未完整核验</t>
         </is>
       </c>
-      <c r="N3" s="64" t="n"/>
-      <c r="O3" s="64" t="inlineStr">
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr">
         <is>
           <t>Apple官方岗位页，2026-06-12发布</t>
         </is>
       </c>
-      <c r="P3" s="64" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>Apple Jobs 官方</t>
         </is>
       </c>
-      <c r="Q3" s="64" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>全球消费电子与软硬件一体化顶级外企，iPad硬件与供应链平台价值高</t>
         </is>
       </c>
-      <c r="R3" s="64" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>iPad硬件/运营链路的技术项目管理，预计涉及跨职能工程协作、供应链/制造节点、风险跟踪和项目推进。</t>
         </is>
       </c>
-      <c r="S3" s="64" t="inlineStr">
+      <c r="S3" t="inlineStr">
         <is>
           <t>正式TPM可能要求多年经验；非纯产品经理；英文和硬件工程语境要求高，需二次确认。</t>
         </is>
       </c>
-      <c r="T3" s="64" t="inlineStr">
+      <c r="T3" t="inlineStr">
         <is>
           <t>英文风险中高；代码风险低；驻厂/供应链沟通风险中。</t>
         </is>
       </c>
-      <c r="U3" s="64" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t>Apple官方搜索页可核验标题、发布时间、地点和Role Number；详情页JS渲染，职责需二次确认</t>
         </is>
       </c>
-      <c r="V3" s="64" t="inlineStr">
+      <c r="V3" t="inlineStr">
         <is>
           <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；非招聘软件或页面未公开HR活跃状态</t>
         </is>
       </c>
-      <c r="W3" s="64" t="inlineStr">
+      <c r="W3" t="inlineStr">
         <is>
           <t>2026-06-17</t>
         </is>
       </c>
-      <c r="X3" s="64" t="inlineStr">
+      <c r="X3" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="Y3" s="64" t="inlineStr">
+      <c r="Y3" t="inlineStr">
         <is>
           <t>Apple智能硬件/TPM版：突出硬件产品、项目协作、NPI/供应链理解、CMF与软硬件结合项目。</t>
         </is>
       </c>
-      <c r="Z3" s="64" t="inlineStr">
+      <c r="Z3" t="inlineStr">
         <is>
           <t>中高</t>
         </is>
       </c>
-      <c r="AA3" s="17" t="inlineStr">
+      <c r="AA3" s="50" t="inlineStr">
         <is>
           <t>https://jobs.apple.com/en-us/details/200666248-3435/technical-program-manager-ipad?team=OPMFG</t>
         </is>
       </c>
-      <c r="AB3" s="64" t="inlineStr">
+      <c r="AB3" s="53" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="AC3" s="64" t="n">
+      <c r="AC3" s="2" t="n">
         <v>79</v>
       </c>
-      <c r="AD3" s="64" t="inlineStr">
+      <c r="AD3" s="2" t="inlineStr">
         <is>
           <t>B档，79分；字段显示主线为主线A-AI终端/智能硬件/TPM/NPI，匹配度中高，原申请优先级P3二次确认后投递。城市/薪资为深圳、Apple官网未公开，薪资匹配为薪资未知；Apple平台价值高，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：全球消费电子与软硬件一体化顶级外企，iPad硬件与供应链平台价值高；JD与可信度为Apple官方搜索页可核验标题、发…、中高，次选表但仍按平台和方向重新排序。关键风险：薪资待确认；JD不精确；英文/粤语/IANG；招聘状态不稳。</t>
         </is>
       </c>
-      <c r="AE3" s="64" t="inlineStr">
+      <c r="AE3" s="2" t="inlineStr">
         <is>
           <t>二次核验后投</t>
         </is>
       </c>
-      <c r="AF3" s="64" t="inlineStr">
+      <c r="AF3" s="2" t="inlineStr">
         <is>
           <t>薪资待确认；JD不精确；英文/粤语/IANG；招聘状态不稳</t>
         </is>
       </c>
-      <c r="AG3" s="64" t="inlineStr">
+      <c r="AG3" s="2" t="inlineStr">
         <is>
           <t>Apple智能硬件/TPM版：突出硬件产品、项目协作、NPI/供应链理解、CMF与软硬件结合项目。</t>
         </is>
@@ -15095,7 +15095,7 @@
       </c>
       <c r="V4" s="48" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接无法精确确认（403），需二次确认；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
         </is>
       </c>
       <c r="W4" s="48" t="inlineStr">
@@ -15142,11 +15142,11 @@
         </is>
       </c>
       <c r="AF4" s="2" t="n">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="AG4" s="2" t="inlineStr">
         <is>
-          <t>B档，71分；字段显示主线为主线A-AIoT/AI终端/软硬件产品，匹配度中，原申请优先级P3次选验证。城市/薪资为香港、未写，薪资匹配为待确认，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：香港线上生活服务与医疗预约平台；JD与可信度为转载/聚合线索、中，次选表但仍按平台和方向重新排序。关键风险：详情或任职要求含3年及以上/3-5年经验门槛，正式主表降为次选复核；薪资待确认；JD不精确；英文/粤语/IANG；出差/驻厂；招聘状态不稳。</t>
+          <t>B档，75分；字段显示主线为主线A-AIoT/AI终端/软硬件产品，匹配度中，原申请优先级P3次选验证。城市/薪资为香港、未写，薪资匹配为待确认，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：香港线上生活服务与医疗预约平台；JD与可信度为转载/聚合线索、中，次选表但仍按平台和方向重新排序。关键风险：详情或任职要求含3年及以上/3-5年经验门槛，正式主表降为次选复核；薪资待确认；JD不精确；英文/粤语/IANG；出差/驻厂。</t>
         </is>
       </c>
       <c r="AH4" s="2" t="inlineStr">
@@ -15156,7 +15156,7 @@
       </c>
       <c r="AI4" s="2" t="inlineStr">
         <is>
-          <t>详情或任职要求含3年及以上/3-5年经验门槛，正式主表降为次选复核；薪资待确认；JD不精确；英文/粤语/IANG；出差/驻厂；招聘状态不稳</t>
+          <t>详情或任职要求含3年及以上/3-5年经验门槛，正式主表降为次选复核；薪资待确认；JD不精确；英文/粤语/IANG；出差/驻厂</t>
         </is>
       </c>
       <c r="AJ4" s="2" t="inlineStr">
@@ -15273,7 +15273,7 @@
       </c>
       <c r="V5" s="47" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接无法精确确认（403），需二次确认；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
         </is>
       </c>
       <c r="W5" s="47" t="inlineStr">
@@ -15320,11 +15320,11 @@
         </is>
       </c>
       <c r="AF5" s="2" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="AG5" s="2" t="inlineStr">
         <is>
-          <t>B档，72分；字段显示主线为主线A-AIoT/AI终端/软硬件产品，匹配度中，原申请优先级P3次选验证。城市/薪资为香港、44k-53k 港币/月，薪资匹配为达标，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：世界500强与全球大型医疗健康集团；JD与可信度为转载/聚合线索、中，次选表但仍按平台和方向重新排序。关键风险：JD不精确；英文/粤语/IANG；出差/驻厂；销售化；招聘状态不稳。</t>
+          <t>B档，74分；字段显示主线为主线A-AIoT/AI终端/软硬件产品，匹配度中，原申请优先级P3次选验证。城市/薪资为香港、44k-53k 港币/月，薪资匹配为达标，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：世界500强与全球大型医疗健康集团；JD与可信度为转载/聚合线索、中，次选表但仍按平台和方向重新排序。关键风险：JD不精确；英文/粤语/IANG；出差/驻厂；销售化。</t>
         </is>
       </c>
       <c r="AH5" s="2" t="inlineStr">
@@ -15334,7 +15334,7 @@
       </c>
       <c r="AI5" s="2" t="inlineStr">
         <is>
-          <t>JD不精确；英文/粤语/IANG；出差/驻厂；销售化；招聘状态不稳</t>
+          <t>JD不精确；英文/粤语/IANG；出差/驻厂；销售化</t>
         </is>
       </c>
       <c r="AJ5" s="2" t="inlineStr">
@@ -15451,7 +15451,7 @@
       </c>
       <c r="V6" s="48" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接无法精确确认（403），需二次确认；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
         </is>
       </c>
       <c r="W6" s="48" t="inlineStr">
@@ -15498,11 +15498,11 @@
         </is>
       </c>
       <c r="AF6" s="2" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="AG6" s="2" t="inlineStr">
         <is>
-          <t>B档，65分；字段显示主线为主线A-AIoT/AI终端/软硬件产品，匹配度中，原申请优先级P3次选验证。城市/薪资为香港、未写，薪资匹配为待确认，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：全球大型保险集团在港核心市场；JD与可信度为转载/聚合线索、中，次选表但仍按平台和方向重新排序。关键风险：详情或任职要求含3年及以上/3-5年经验门槛，正式主表降为次选复核；薪资待确认；JD不精确；英文/粤语/IANG；出差/驻厂；销售化；招聘状态不稳。</t>
+          <t>B档，67分；字段显示主线为主线A-AIoT/AI终端/软硬件产品，匹配度中，原申请优先级P3次选验证。城市/薪资为香港、未写，薪资匹配为待确认，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：全球大型保险集团在港核心市场；JD与可信度为转载/聚合线索、中，次选表但仍按平台和方向重新排序。关键风险：详情或任职要求含3年及以上/3-5年经验门槛，正式主表降为次选复核；薪资待确认；JD不精确；英文/粤语/IANG；出差/驻厂；销售化。</t>
         </is>
       </c>
       <c r="AH6" s="2" t="inlineStr">
@@ -15512,7 +15512,7 @@
       </c>
       <c r="AI6" s="2" t="inlineStr">
         <is>
-          <t>详情或任职要求含3年及以上/3-5年经验门槛，正式主表降为次选复核；薪资待确认；JD不精确；英文/粤语/IANG；出差/驻厂；销售化；招聘状态不稳</t>
+          <t>详情或任职要求含3年及以上/3-5年经验门槛，正式主表降为次选复核；薪资待确认；JD不精确；英文/粤语/IANG；出差/驻厂；销售化</t>
         </is>
       </c>
       <c r="AJ6" s="2" t="inlineStr">
@@ -15629,7 +15629,7 @@
       </c>
       <c r="V7" s="47" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接无法精确确认（403），需二次确认；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
         </is>
       </c>
       <c r="W7" s="47" t="inlineStr">
@@ -15676,11 +15676,11 @@
         </is>
       </c>
       <c r="AF7" s="2" t="n">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="AG7" s="2" t="inlineStr">
         <is>
-          <t>B档，65分；字段显示主线为主线A-AIoT/AI终端/软硬件产品，匹配度中，原申请优先级P3次选验证。城市/薪资为香港、未写，薪资匹配为待确认，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：香港大型餐饮与零售集团；JD与可信度为转载/聚合线索、中，次选表但仍按平台和方向重新排序。关键风险：详情或任职要求含3年及以上/3-5年经验门槛，正式主表降为次选复核；薪资待确认；JD不精确；英文/粤语/IANG；出差/驻厂；招聘状态不稳。</t>
+          <t>B档，69分；字段显示主线为主线A-AIoT/AI终端/软硬件产品，匹配度中，原申请优先级P3次选验证。城市/薪资为香港、未写，薪资匹配为待确认，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：香港大型餐饮与零售集团；JD与可信度为转载/聚合线索、中，次选表但仍按平台和方向重新排序。关键风险：详情或任职要求含3年及以上/3-5年经验门槛，正式主表降为次选复核；薪资待确认；JD不精确；英文/粤语/IANG；出差/驻厂。</t>
         </is>
       </c>
       <c r="AH7" s="2" t="inlineStr">
@@ -15690,7 +15690,7 @@
       </c>
       <c r="AI7" s="2" t="inlineStr">
         <is>
-          <t>详情或任职要求含3年及以上/3-5年经验门槛，正式主表降为次选复核；薪资待确认；JD不精确；英文/粤语/IANG；出差/驻厂；招聘状态不稳</t>
+          <t>详情或任职要求含3年及以上/3-5年经验门槛，正式主表降为次选复核；薪资待确认；JD不精确；英文/粤语/IANG；出差/驻厂</t>
         </is>
       </c>
       <c r="AJ7" s="2" t="inlineStr">
@@ -15985,7 +15985,7 @@
       </c>
       <c r="V9" s="47" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接无法精确确认（403），需二次确认；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
         </is>
       </c>
       <c r="W9" s="47" t="inlineStr">
@@ -16032,11 +16032,11 @@
         </is>
       </c>
       <c r="AF9" s="2" t="n">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="AG9" s="2" t="inlineStr">
         <is>
-          <t>B档，65分；字段显示主线为主线A-AIoT/AI终端/软硬件产品，匹配度中，原申请优先级P3次选验证。城市/薪资为香港、未写，薪资匹配为待确认，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：香港大型贸易分销与汽车消费品集团；JD与可信度为转载/聚合线索、中，次选表但仍按平台和方向重新排序。关键风险：详情或任职要求含3年及以上/3-5年经验门槛，正式主表降为次选复核；薪资待确认；JD不精确；英文/粤语/IANG；出差/驻厂；招聘状态不稳。</t>
+          <t>B档，69分；字段显示主线为主线A-AIoT/AI终端/软硬件产品，匹配度中，原申请优先级P3次选验证。城市/薪资为香港、未写，薪资匹配为待确认，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：香港大型贸易分销与汽车消费品集团；JD与可信度为转载/聚合线索、中，次选表但仍按平台和方向重新排序。关键风险：详情或任职要求含3年及以上/3-5年经验门槛，正式主表降为次选复核；薪资待确认；JD不精确；英文/粤语/IANG；出差/驻厂。</t>
         </is>
       </c>
       <c r="AH9" s="2" t="inlineStr">
@@ -16046,7 +16046,7 @@
       </c>
       <c r="AI9" s="2" t="inlineStr">
         <is>
-          <t>详情或任职要求含3年及以上/3-5年经验门槛，正式主表降为次选复核；薪资待确认；JD不精确；英文/粤语/IANG；出差/驻厂；招聘状态不稳</t>
+          <t>详情或任职要求含3年及以上/3-5年经验门槛，正式主表降为次选复核；薪资待确认；JD不精确；英文/粤语/IANG；出差/驻厂</t>
         </is>
       </c>
       <c r="AJ9" s="2" t="inlineStr">
@@ -16163,7 +16163,7 @@
       </c>
       <c r="V10" s="48" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接无法精确确认（403），需二次确认；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
         </is>
       </c>
       <c r="W10" s="48" t="inlineStr">
@@ -16210,11 +16210,11 @@
         </is>
       </c>
       <c r="AF10" s="2" t="n">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="AG10" s="2" t="inlineStr">
         <is>
-          <t>B档，71分；字段显示主线为主线A-AIoT/AI终端/软硬件产品，匹配度中，原申请优先级P3次选验证。城市/薪资为香港、未写，薪资匹配为待确认，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：香港快消外企与知名品牌集团；JD与可信度为转载/聚合线索、中，次选表但仍按平台和方向重新排序。关键风险：详情或任职要求含3年及以上/3-5年经验门槛，正式主表降为次选复核；薪资待确认；JD不精确；英文/粤语/IANG；出差/驻厂；招聘状态不稳。</t>
+          <t>B档，75分；字段显示主线为主线A-AIoT/AI终端/软硬件产品，匹配度中，原申请优先级P3次选验证。城市/薪资为香港、未写，薪资匹配为待确认，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：香港快消外企与知名品牌集团；JD与可信度为转载/聚合线索、中，次选表但仍按平台和方向重新排序。关键风险：详情或任职要求含3年及以上/3-5年经验门槛，正式主表降为次选复核；薪资待确认；JD不精确；英文/粤语/IANG；出差/驻厂。</t>
         </is>
       </c>
       <c r="AH10" s="2" t="inlineStr">
@@ -16224,7 +16224,7 @@
       </c>
       <c r="AI10" s="2" t="inlineStr">
         <is>
-          <t>详情或任职要求含3年及以上/3-5年经验门槛，正式主表降为次选复核；薪资待确认；JD不精确；英文/粤语/IANG；出差/驻厂；招聘状态不稳</t>
+          <t>详情或任职要求含3年及以上/3-5年经验门槛，正式主表降为次选复核；薪资待确认；JD不精确；英文/粤语/IANG；出差/驻厂</t>
         </is>
       </c>
       <c r="AJ10" s="2" t="inlineStr">
@@ -16341,7 +16341,7 @@
       </c>
       <c r="V11" s="47" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接无法精确确认（403），需二次确认；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
         </is>
       </c>
       <c r="W11" s="47" t="inlineStr">
@@ -16388,11 +16388,11 @@
         </is>
       </c>
       <c r="AF11" s="2" t="n">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="AG11" s="2" t="inlineStr">
         <is>
-          <t>B档，71分；字段显示主线为主线A-AIoT/AI终端/软硬件产品，匹配度中，原申请优先级P3次选验证。城市/薪资为香港、未写，薪资匹配为待确认，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：香港消费电子与电商零售品牌；JD与可信度为转载/聚合线索、中，次选表但仍按平台和方向重新排序。关键风险：详情或任职要求含3年及以上/3-5年经验门槛，正式主表降为次选复核；薪资待确认；JD不精确；英文/粤语/IANG；出差/驻厂；招聘状态不稳。</t>
+          <t>B档，75分；字段显示主线为主线A-AIoT/AI终端/软硬件产品，匹配度中，原申请优先级P3次选验证。城市/薪资为香港、未写，薪资匹配为待确认，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：香港消费电子与电商零售品牌；JD与可信度为转载/聚合线索、中，次选表但仍按平台和方向重新排序。关键风险：详情或任职要求含3年及以上/3-5年经验门槛，正式主表降为次选复核；薪资待确认；JD不精确；英文/粤语/IANG；出差/驻厂。</t>
         </is>
       </c>
       <c r="AH11" s="2" t="inlineStr">
@@ -16402,7 +16402,7 @@
       </c>
       <c r="AI11" s="2" t="inlineStr">
         <is>
-          <t>详情或任职要求含3年及以上/3-5年经验门槛，正式主表降为次选复核；薪资待确认；JD不精确；英文/粤语/IANG；出差/驻厂；招聘状态不稳</t>
+          <t>详情或任职要求含3年及以上/3-5年经验门槛，正式主表降为次选复核；薪资待确认；JD不精确；英文/粤语/IANG；出差/驻厂</t>
         </is>
       </c>
       <c r="AJ11" s="2" t="inlineStr">
@@ -16519,7 +16519,7 @@
       </c>
       <c r="V12" s="47" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接无法精确确认（403），需二次确认；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
         </is>
       </c>
       <c r="W12" s="47" t="inlineStr">
@@ -16566,11 +16566,11 @@
         </is>
       </c>
       <c r="AF12" s="2" t="n">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="AG12" s="2" t="inlineStr">
         <is>
-          <t>B档，65分；字段显示主线为主线A-AIoT/AI终端/软硬件产品，匹配度中，原申请优先级P3次选验证。城市/薪资为香港、未写，薪资匹配为待确认，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：香港持牌银行与台湾金控系机构；JD与可信度为转载/聚合线索、中，次选表但仍按平台和方向重新排序。关键风险：薪资待确认；JD不精确；英文/粤语/IANG；出差/驻厂；招聘状态不稳。</t>
+          <t>B档，69分；字段显示主线为主线A-AIoT/AI终端/软硬件产品，匹配度中，原申请优先级P3次选验证。城市/薪资为香港、未写，薪资匹配为待确认，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：香港持牌银行与台湾金控系机构；JD与可信度为转载/聚合线索、中，次选表但仍按平台和方向重新排序。关键风险：薪资待确认；JD不精确；英文/粤语/IANG；出差/驻厂。</t>
         </is>
       </c>
       <c r="AH12" s="2" t="inlineStr">
@@ -16580,7 +16580,7 @@
       </c>
       <c r="AI12" s="2" t="inlineStr">
         <is>
-          <t>薪资待确认；JD不精确；英文/粤语/IANG；出差/驻厂；招聘状态不稳</t>
+          <t>薪资待确认；JD不精确；英文/粤语/IANG；出差/驻厂</t>
         </is>
       </c>
       <c r="AJ12" s="2" t="inlineStr">
@@ -16875,7 +16875,7 @@
       </c>
       <c r="V14" s="48" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接无法精确确认（403），需二次确认；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
         </is>
       </c>
       <c r="W14" s="48" t="inlineStr">
@@ -16922,11 +16922,11 @@
         </is>
       </c>
       <c r="AF14" s="2" t="n">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="AG14" s="2" t="inlineStr">
         <is>
-          <t>B档，71分；字段显示主线为主线A-AIoT/AI终端/软硬件产品，匹配度中，原申请优先级P3次选验证。城市/薪资为香港、未写，薪资匹配为待确认，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：全球顶级学术出版机构；JD与可信度为转载/聚合线索、中，次选表但仍按平台和方向重新排序。关键风险：详情或任职要求含3年及以上/3-5年经验门槛，正式主表降为次选复核；薪资待确认；JD不精确；英文/粤语/IANG；出差/驻厂；招聘状态不稳。</t>
+          <t>B档，75分；字段显示主线为主线A-AIoT/AI终端/软硬件产品，匹配度中，原申请优先级P3次选验证。城市/薪资为香港、未写，薪资匹配为待确认，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：全球顶级学术出版机构；JD与可信度为转载/聚合线索、中，次选表但仍按平台和方向重新排序。关键风险：详情或任职要求含3年及以上/3-5年经验门槛，正式主表降为次选复核；薪资待确认；JD不精确；英文/粤语/IANG；出差/驻厂。</t>
         </is>
       </c>
       <c r="AH14" s="2" t="inlineStr">
@@ -16936,7 +16936,7 @@
       </c>
       <c r="AI14" s="2" t="inlineStr">
         <is>
-          <t>详情或任职要求含3年及以上/3-5年经验门槛，正式主表降为次选复核；薪资待确认；JD不精确；英文/粤语/IANG；出差/驻厂；招聘状态不稳</t>
+          <t>详情或任职要求含3年及以上/3-5年经验门槛，正式主表降为次选复核；薪资待确认；JD不精确；英文/粤语/IANG；出差/驻厂</t>
         </is>
       </c>
       <c r="AJ14" s="2" t="inlineStr">
@@ -22393,7 +22393,7 @@
       </c>
       <c r="V45" s="48" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接无法精确确认（429），需二次确认；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
         </is>
       </c>
       <c r="W45" s="48" t="inlineStr">
@@ -22444,7 +22444,7 @@
       </c>
       <c r="AG45" s="2" t="inlineStr">
         <is>
-          <t>B档，79分；字段显示主线为主线A-AIoT/AI终端/软硬件产品，匹配度中高，原申请优先级P3次选验证。城市/薪资为香港、未写，薪资匹配为不适用，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：香港商户收单与支付科技公司；JD与可信度为精确JD、高，次选表但仍按平台和方向重新排序。关键风险：英文/粤语/IANG；出差/驻厂；招聘状态不稳。</t>
+          <t>B档，79分；字段显示主线为主线A-AIoT/AI终端/软硬件产品，匹配度中高，原申请优先级P3次选验证。城市/薪资为香港、未写，薪资匹配为不适用，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：香港商户收单与支付科技公司；JD与可信度为精确JD、高，次选表但仍按平台和方向重新排序。关键风险：英文/粤语/IANG；出差/驻厂。</t>
         </is>
       </c>
       <c r="AH45" s="2" t="inlineStr">
@@ -22454,7 +22454,7 @@
       </c>
       <c r="AI45" s="2" t="inlineStr">
         <is>
-          <t>英文/粤语/IANG；出差/驻厂；招聘状态不稳</t>
+          <t>英文/粤语/IANG；出差/驻厂</t>
         </is>
       </c>
       <c r="AJ45" s="2" t="inlineStr">
@@ -22749,7 +22749,7 @@
       </c>
       <c r="V47" s="48" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接无法精确确认（429），需二次确认；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
         </is>
       </c>
       <c r="W47" s="48" t="inlineStr">
@@ -22800,7 +22800,7 @@
       </c>
       <c r="AG47" s="2" t="inlineStr">
         <is>
-          <t>B档，79分；字段显示主线为主线A-AIoT/AI终端/软硬件产品，匹配度中高，原申请优先级P3次选验证。城市/薪资为香港、未写，薪资匹配为不适用，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：AI 产品创业公司；JD与可信度为精确JD、高，次选表但仍按平台和方向重新排序。关键风险：英文/粤语/IANG；出差/驻厂；招聘状态不稳。</t>
+          <t>B档，79分；字段显示主线为主线A-AIoT/AI终端/软硬件产品，匹配度中高，原申请优先级P3次选验证。城市/薪资为香港、未写，薪资匹配为不适用，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：AI 产品创业公司；JD与可信度为精确JD、高，次选表但仍按平台和方向重新排序。关键风险：英文/粤语/IANG；出差/驻厂。</t>
         </is>
       </c>
       <c r="AH47" s="2" t="inlineStr">
@@ -22810,7 +22810,7 @@
       </c>
       <c r="AI47" s="2" t="inlineStr">
         <is>
-          <t>英文/粤语/IANG；出差/驻厂；招聘状态不稳</t>
+          <t>英文/粤语/IANG；出差/驻厂</t>
         </is>
       </c>
       <c r="AJ47" s="2" t="inlineStr">
@@ -23105,7 +23105,7 @@
       </c>
       <c r="V49" s="48" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接无法精确确认（429），需二次确认；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
         </is>
       </c>
       <c r="W49" s="48" t="inlineStr">
@@ -23156,7 +23156,7 @@
       </c>
       <c r="AG49" s="2" t="inlineStr">
         <is>
-          <t>B档，79分；字段显示主线为主线A-AIoT/AI终端/软硬件产品，匹配度中，原申请优先级P3次选验证。城市/薪资为香港、未写，薪资匹配为不适用，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：全球玩具与娱乐大厂；JD与可信度为精确JD、高，次选表但仍按平台和方向重新排序。关键风险：英文/粤语/IANG；出差/驻厂；招聘状态不稳。</t>
+          <t>B档，79分；字段显示主线为主线A-AIoT/AI终端/软硬件产品，匹配度中，原申请优先级P3次选验证。城市/薪资为香港、未写，薪资匹配为不适用，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：全球玩具与娱乐大厂；JD与可信度为精确JD、高，次选表但仍按平台和方向重新排序。关键风险：英文/粤语/IANG；出差/驻厂。</t>
         </is>
       </c>
       <c r="AH49" s="2" t="inlineStr">
@@ -23166,7 +23166,7 @@
       </c>
       <c r="AI49" s="2" t="inlineStr">
         <is>
-          <t>英文/粤语/IANG；出差/驻厂；招聘状态不稳</t>
+          <t>英文/粤语/IANG；出差/驻厂</t>
         </is>
       </c>
       <c r="AJ49" s="2" t="inlineStr">
@@ -24018,7 +24018,7 @@
           <t>高</t>
         </is>
       </c>
-      <c r="AA54" s="17" t="inlineStr">
+      <c r="AA54" s="62" t="inlineStr">
         <is>
           <t>https://jobs.apple.com/en-us/details/200658508-3435/product-design-engineer-mechanical?team=HRDWR</t>
         </is>
@@ -24196,7 +24196,7 @@
           <t>高</t>
         </is>
       </c>
-      <c r="AA55" s="17" t="inlineStr">
+      <c r="AA55" s="62" t="inlineStr">
         <is>
           <t>https://jobs.apple.com/en-us/details/200644919-3435/manufacturing-design-engineer-intern-shenzhen-changsha?team=STDNT</t>
         </is>
@@ -25415,7 +25415,7 @@
       </c>
       <c r="V62" s="48" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
+          <t>2026-06-17 自动复核：链接无法精确确认（429），需二次确认；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
         </is>
       </c>
       <c r="W62" s="48" t="inlineStr">
@@ -25462,7 +25462,7 @@
       </c>
       <c r="AG62" s="2" t="inlineStr">
         <is>
-          <t>B档，79分；字段显示主线为主线B-AI应用落地/FDE/GenAI部署，匹配度中高，原申请优先级P2验证（FDE上限岗位）。城市/薪资为香港（可选 Taipei；投前…、官方未公开，薪资匹配为待确认；平台/方向强，香港薪资上限…，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：全球云与AI平台头部公司；Google Cloud企业级AI与云服务；JD与可信度为精确JD（LinkedIn公共页完…、高，次选表但仍按平台和方向重新排序。关键风险：薪资待确认；英文/粤语/IANG；代码/技术面。</t>
+          <t>B档，79分；字段显示主线为主线B-AI应用落地/FDE/GenAI部署，匹配度中高，原申请优先级P2验证（FDE上限岗位）。城市/薪资为香港（可选 Taipei；投前…、官方未公开，薪资匹配为待确认；平台/方向强，香港薪资上限…，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：全球云与AI平台头部公司；Google Cloud企业级AI与云服务；JD与可信度为精确JD（LinkedIn公共页完…、高，次选表但仍按平台和方向重新排序。关键风险：薪资待确认；英文/粤语/IANG；代码/技术面；招聘状态不稳。</t>
         </is>
       </c>
       <c r="AH62" s="2" t="inlineStr">
@@ -25472,7 +25472,7 @@
       </c>
       <c r="AI62" s="2" t="inlineStr">
         <is>
-          <t>薪资待确认；英文/粤语/IANG；代码/技术面</t>
+          <t>薪资待确认；英文/粤语/IANG；代码/技术面；招聘状态不稳</t>
         </is>
       </c>
       <c r="AJ62" s="2" t="inlineStr">
@@ -26301,7 +26301,7 @@
       </c>
       <c r="V67" s="48" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；非招聘软件或页面未公开HR活跃状态</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；非招聘软件或页面未公开HR活跃状态</t>
         </is>
       </c>
       <c r="W67" s="48" t="inlineStr">
@@ -26479,7 +26479,7 @@
       </c>
       <c r="V68" s="48" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；非招聘软件或页面未公开HR活跃状态</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；非招聘软件或页面未公开HR活跃状态</t>
         </is>
       </c>
       <c r="W68" s="48" t="inlineStr">
@@ -29144,7 +29144,7 @@
           <t>中高</t>
         </is>
       </c>
-      <c r="AA83" s="17" t="inlineStr">
+      <c r="AA83" s="62" t="inlineStr">
         <is>
           <t>https://jobs.apple.com/en-us/details/200666248-3435/technical-program-manager-ipad?team=OPMFG</t>
         </is>
@@ -29991,7 +29991,7 @@
       </c>
       <c r="V88" s="47" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；非招聘软件或页面未公开HR活跃状态</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；公开可见HR活跃状态：刚刚活跃</t>
         </is>
       </c>
       <c r="W88" s="47" t="inlineStr">
@@ -30821,7 +30821,7 @@
       </c>
       <c r="Q4" s="47" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；非招聘软件或页面未公开HR活跃状态</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；非招聘软件或页面未公开HR活跃状态</t>
         </is>
       </c>
       <c r="R4" s="47" t="inlineStr">
@@ -31151,7 +31151,7 @@
       </c>
       <c r="Q6" s="47" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；非招聘软件或页面未公开HR活跃状态</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；非招聘软件或页面未公开HR活跃状态</t>
         </is>
       </c>
       <c r="R6" s="47" t="inlineStr">
@@ -31811,7 +31811,7 @@
       </c>
       <c r="Q10" s="48" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接无法精确确认（429），需二次确认；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
         </is>
       </c>
       <c r="R10" s="48" t="inlineStr">
@@ -31870,21 +31870,21 @@
         </is>
       </c>
       <c r="AC10" s="2" t="n">
-        <v>87</v>
+        <v>98</v>
       </c>
       <c r="AD10" s="2" t="inlineStr">
         <is>
-          <t>A档，87分；字段显示主线为备线C-AI解决方案/数字化产品，匹配度中高，原申请优先级P3练手/备选实习。城市/薪资为深圳、未写，薪资匹配为实习可接受，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：腾讯云CSIG，中国头部云与产业互联网平台，做云、AI、安全和行业数字化；JD与可信度为精确JD、高，入池岗位。关键风险：出差/驻厂；招聘状态不稳。</t>
+          <t>A档，98分；字段显示主线为备线C-AI解决方案/数字化产品，匹配度中高，原申请优先级P3练手/备选实习。城市/薪资为深圳、未写，薪资匹配为实习可接受，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：腾讯云CSIG，中国头部云与产业互联网平台，做云、AI、安全和行业数字化；JD与可信度为精确JD、高，入池岗位。关键风险：出差/驻厂。</t>
         </is>
       </c>
       <c r="AE10" s="2" t="inlineStr">
         <is>
-          <t>先核验再投</t>
+          <t>定制简历后优先投</t>
         </is>
       </c>
       <c r="AF10" s="2" t="inlineStr">
         <is>
-          <t>出差/驻厂；招聘状态不稳</t>
+          <t>出差/驻厂</t>
         </is>
       </c>
       <c r="AG10" s="2" t="inlineStr">
@@ -32471,7 +32471,7 @@
       </c>
       <c r="Q14" s="47" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
         </is>
       </c>
       <c r="R14" s="47" t="inlineStr">
@@ -32801,7 +32801,7 @@
       </c>
       <c r="Q16" s="47" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
         </is>
       </c>
       <c r="R16" s="47" t="inlineStr">
@@ -33296,7 +33296,7 @@
       </c>
       <c r="Q19" s="48" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
         </is>
       </c>
       <c r="R19" s="48" t="inlineStr">
@@ -35276,7 +35276,7 @@
       </c>
       <c r="Q31" s="47" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接无法精确确认（429），需二次确认；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
         </is>
       </c>
       <c r="R31" s="47" t="inlineStr">
@@ -35339,17 +35339,17 @@
       </c>
       <c r="AD31" s="2" t="inlineStr">
         <is>
-          <t>C档，50分；字段显示主线为主线A-AIoT/AI终端/软硬件产品，匹配度高，原申请优先级P3次选验证。城市/薪资为香港、未写，薪资匹配为待确认，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：全球外设龙头与瑞士国际品牌；JD与可信度为精确JD、高，入池岗位。关键风险：资深/高年限硬门槛：标题含高级/资深/专家/负责人/Lead/Owner等资深信号；薪资待确认；英文/粤语/IANG；出差/驻厂；招聘状态不稳。</t>
+          <t>C档，50分；字段显示主线为主线A-AIoT/AI终端/软硬件产品，匹配度高，原申请优先级P3次选验证。城市/薪资为香港、未写，薪资匹配为待确认，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：全球外设龙头与瑞士国际品牌；JD与可信度为精确JD、高，入池岗位。关键风险：资深/高年限硬门槛：标题含高级/资深/专家/负责人/Lead/Owner等资深信号；薪资待确认；英文/粤语/IANG；出差/驻厂。</t>
         </is>
       </c>
       <c r="AE31" s="2" t="inlineStr">
         <is>
-          <t>观察</t>
+          <t>练手投/暂缓</t>
         </is>
       </c>
       <c r="AF31" s="2" t="inlineStr">
         <is>
-          <t>资深/高年限硬门槛：标题含高级/资深/专家/负责人/Lead/Owner等资深信号；薪资待确认；英文/粤语/IANG；出差/驻厂；招聘状态不稳</t>
+          <t>资深/高年限硬门槛：标题含高级/资深/专家/负责人/Lead/Owner等资深信号；薪资待确认；英文/粤语/IANG；出差/驻厂</t>
         </is>
       </c>
       <c r="AG31" s="2" t="inlineStr">
@@ -38246,7 +38246,7 @@
       </c>
       <c r="Q49" s="47" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接无法精确确认（429），需二次确认；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
         </is>
       </c>
       <c r="R49" s="47" t="inlineStr">
@@ -38305,11 +38305,11 @@
         </is>
       </c>
       <c r="AC49" s="2" t="n">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="AD49" s="2" t="inlineStr">
         <is>
-          <t>B档，69分；字段显示主线为主线B-AI应用落地/AI产品工程师，匹配度中高，原申请优先级P2AI应用实习。城市/薪资为香港/深圳、未公开，薪资匹配为实习可接受，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：移动设备管理、远程控制和跨设备协同工具公司，香港/深圳协同；JD与可信度为入口页/搜索页、中高，入池岗位。关键风险：薪资待确认；JD不精确；英文/粤语/IANG；出差/驻厂；招聘状态不稳。</t>
+          <t>B档，73分；字段显示主线为主线B-AI应用落地/AI产品工程师，匹配度中高，原申请优先级P2AI应用实习。城市/薪资为香港/深圳、未公开，薪资匹配为实习可接受，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：移动设备管理、远程控制和跨设备协同工具公司，香港/深圳协同；JD与可信度为入口页/搜索页、中高，入池岗位。关键风险：薪资待确认；JD不精确；英文/粤语/IANG；出差/驻厂。</t>
         </is>
       </c>
       <c r="AE49" s="2" t="inlineStr">
@@ -38319,7 +38319,7 @@
       </c>
       <c r="AF49" s="2" t="inlineStr">
         <is>
-          <t>薪资待确认；JD不精确；英文/粤语/IANG；出差/驻厂；招聘状态不稳</t>
+          <t>薪资待确认；JD不精确；英文/粤语/IANG；出差/驻厂</t>
         </is>
       </c>
       <c r="AG49" s="2" t="inlineStr">
@@ -39236,7 +39236,7 @@
       </c>
       <c r="Q55" s="48" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接无法精确确认（429），需二次确认；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
         </is>
       </c>
       <c r="R55" s="48" t="inlineStr">
@@ -39299,7 +39299,7 @@
       </c>
       <c r="AD55" s="2" t="inlineStr">
         <is>
-          <t>B档，79分；字段显示主线为主线A-AIoT/AI终端/软硬件产品，匹配度高，原申请优先级P1主线实习。城市/薪资为深圳、400-500/天待确认，薪资匹配为实习可接受，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：深圳创客硬件和桌面激光加工设备出海品牌，软硬件结合和创作者生态强；JD与可信度为入口页/搜索页、中高，入池岗位。关键风险：薪资待确认；JD不精确；出差/驻厂；招聘状态不稳。</t>
+          <t>B档，79分；字段显示主线为主线A-AIoT/AI终端/软硬件产品，匹配度高，原申请优先级P1主线实习。城市/薪资为深圳、400-500/天待确认，薪资匹配为实习可接受，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：深圳创客硬件和桌面激光加工设备出海品牌，软硬件结合和创作者生态强；JD与可信度为入口页/搜索页、中高，入池岗位。关键风险：薪资待确认；JD不精确；出差/驻厂。</t>
         </is>
       </c>
       <c r="AE55" s="2" t="inlineStr">
@@ -39309,7 +39309,7 @@
       </c>
       <c r="AF55" s="2" t="inlineStr">
         <is>
-          <t>薪资待确认；JD不精确；出差/驻厂；招聘状态不稳</t>
+          <t>薪资待确认；JD不精确；出差/驻厂</t>
         </is>
       </c>
       <c r="AG55" s="2" t="inlineStr">
@@ -40721,7 +40721,7 @@
       </c>
       <c r="Q64" s="47" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；非招聘软件或页面未公开HR活跃状态</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；非招聘软件或页面未公开HR活跃状态</t>
         </is>
       </c>
       <c r="R64" s="47" t="inlineStr">
@@ -46146,7 +46146,7 @@
       </c>
       <c r="Q97" s="48" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
+          <t>2026-06-17 自动复核：链接无法精确确认（403），需二次确认；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
         </is>
       </c>
       <c r="R97" s="48" t="inlineStr">
@@ -46205,17 +46205,17 @@
       </c>
       <c r="AD97" s="2" t="inlineStr">
         <is>
-          <t>A档，100分；字段显示主线为主线B-AI应用落地/AI产品工程师，匹配度高，原申请优先级P1主攻。城市/薪资为香港、HK$22,000-28,000/月，薪资匹配为部分达标，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：香港本地Agentic AI平台公司，主打企业客服与销售流程自动化；JD与可信度为中高、中高，入池岗位。关键风险：英文/粤语/IANG。</t>
+          <t>A档，100分；字段显示主线为主线B-AI应用落地/AI产品工程师，匹配度高，原申请优先级P1主攻。城市/薪资为香港、HK$22,000-28,000/月，薪资匹配为部分达标，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：香港本地Agentic AI平台公司，主打企业客服与销售流程自动化；JD与可信度为中高、中高，入池岗位。关键风险：英文/粤语/IANG；招聘状态不稳。</t>
         </is>
       </c>
       <c r="AE97" s="2" t="inlineStr">
         <is>
-          <t>重点准备后投</t>
+          <t>先核验再投</t>
         </is>
       </c>
       <c r="AF97" s="2" t="inlineStr">
         <is>
-          <t>英文/粤语/IANG</t>
+          <t>英文/粤语/IANG；招聘状态不稳</t>
         </is>
       </c>
       <c r="AG97" s="2" t="inlineStr">
@@ -46464,7 +46464,7 @@
       </c>
       <c r="Q99" s="48" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接无法精确确认（403），需二次确认；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
         </is>
       </c>
       <c r="R99" s="48" t="inlineStr">
@@ -46515,11 +46515,11 @@
         </is>
       </c>
       <c r="AC99" s="2" t="n">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="AD99" s="2" t="inlineStr">
         <is>
-          <t>B档，73分；字段显示主线为备线C-AI解决方案/数字化产品，匹配度中高，原申请优先级P2验证。城市/薪资为香港、未写，薪资匹配为待确认，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：香港本地ERP/企业系统厂商，正在把AI/CRM/ERP打包为企业数字化方案；JD与可信度为搜索结果核验、中，扩源入口需后置核验。关键风险：薪资待确认；英文/粤语/IANG；招聘状态不稳。</t>
+          <t>B档，76分；字段显示主线为备线C-AI解决方案/数字化产品，匹配度中高，原申请优先级P2验证。城市/薪资为香港、未写，薪资匹配为待确认，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：香港本地ERP/企业系统厂商，正在把AI/CRM/ERP打包为企业数字化方案；JD与可信度为搜索结果核验、中，扩源入口需后置核验。关键风险：薪资待确认；英文/粤语/IANG。</t>
         </is>
       </c>
       <c r="AE99" s="2" t="inlineStr">
@@ -46529,7 +46529,7 @@
       </c>
       <c r="AF99" s="2" t="inlineStr">
         <is>
-          <t>薪资待确认；英文/粤语/IANG；招聘状态不稳</t>
+          <t>薪资待确认；英文/粤语/IANG</t>
         </is>
       </c>
       <c r="AG99" s="2" t="inlineStr">
@@ -47104,7 +47104,7 @@
       </c>
       <c r="Q103" s="48" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；非招聘软件或页面未公开HR活跃状态</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；公开可见HR活跃状态：刚刚活跃</t>
         </is>
       </c>
       <c r="R103" s="48" t="inlineStr">
@@ -47748,7 +47748,7 @@
       </c>
       <c r="Q107" s="48" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接无法精确确认（403），需二次确认；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
         </is>
       </c>
       <c r="R107" s="48" t="inlineStr">
@@ -47803,11 +47803,11 @@
         </is>
       </c>
       <c r="AC107" s="2" t="n">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="AD107" s="2" t="inlineStr">
         <is>
-          <t>B档，72分；字段显示主线为主线B-AI应用落地/AI产品工程师（偏业务落地与原型实现），匹配度中高，原申请优先级P2验证。城市/薪资为香港-Kowloon Bay、未写，薪资匹配为待确认，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：香港数据中心与IT服务公司，业务覆盖AI Infrastructure、HPC与企…；JD与可信度为搜索结果核验，需二次确认、中，扩源入口需后置核验。关键风险：薪资待确认；英文/粤语/IANG；招聘状态不稳。</t>
+          <t>B档，76分；字段显示主线为主线B-AI应用落地/AI产品工程师（偏业务落地与原型实现），匹配度中高，原申请优先级P2验证。城市/薪资为香港-Kowloon Bay、未写，薪资匹配为待确认，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：香港数据中心与IT服务公司，业务覆盖AI Infrastructure、HPC与企…；JD与可信度为搜索结果核验，需二次确认、中，扩源入口需后置核验。关键风险：薪资待确认；英文/粤语/IANG；招聘状态不稳。</t>
         </is>
       </c>
       <c r="AE107" s="2" t="inlineStr">
@@ -47909,7 +47909,7 @@
       </c>
       <c r="Q108" s="48" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接无法精确确认（403），需二次确认；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
         </is>
       </c>
       <c r="R108" s="48" t="inlineStr">
@@ -48875,7 +48875,7 @@
       </c>
       <c r="Q114" s="48" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
         </is>
       </c>
       <c r="R114" s="48" t="inlineStr">
@@ -52145,7 +52145,7 @@
       </c>
       <c r="Q134" s="47" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；非招聘软件或页面未公开HR活跃状态</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；非招聘软件或页面未公开HR活跃状态</t>
         </is>
       </c>
       <c r="R134" s="47" t="inlineStr">
@@ -52308,7 +52308,7 @@
       </c>
       <c r="Q135" s="47" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；非招聘软件或页面未公开HR活跃状态</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；非招聘软件或页面未公开HR活跃状态</t>
         </is>
       </c>
       <c r="R135" s="47" t="inlineStr">
@@ -52634,7 +52634,7 @@
       </c>
       <c r="Q137" s="47" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；非招聘软件或页面未公开HR活跃状态</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；非招聘软件或页面未公开HR活跃状态</t>
         </is>
       </c>
       <c r="R137" s="47" t="inlineStr">
@@ -52797,7 +52797,7 @@
       </c>
       <c r="Q138" s="47" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；非招聘软件或页面未公开HR活跃状态</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；非招聘软件或页面未公开HR活跃状态</t>
         </is>
       </c>
       <c r="R138" s="47" t="inlineStr">
@@ -52960,7 +52960,7 @@
       </c>
       <c r="Q139" s="47" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；非招聘软件或页面未公开HR活跃状态</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；非招聘软件或页面未公开HR活跃状态</t>
         </is>
       </c>
       <c r="R139" s="47" t="inlineStr">
@@ -54101,7 +54101,7 @@
       </c>
       <c r="Q146" s="47" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；非招聘软件或页面未公开HR活跃状态</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；非招聘软件或页面未公开HR活跃状态</t>
         </is>
       </c>
       <c r="R146" s="47" t="inlineStr">
@@ -54753,7 +54753,7 @@
       </c>
       <c r="Q150" s="47" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；非招聘软件或页面未公开HR活跃状态</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；非招聘软件或页面未公开HR活跃状态</t>
         </is>
       </c>
       <c r="R150" s="47" t="inlineStr">
@@ -56691,7 +56691,7 @@
           <t>中高</t>
         </is>
       </c>
-      <c r="U162" s="17" t="inlineStr">
+      <c r="U162" s="62" t="inlineStr">
         <is>
           <t>https://jobs.apple.com/en-us/details/200494847-3435/engineering-project-manager-intern-shanghai-shenzhen?team=HRDWR</t>
         </is>
@@ -56728,12 +56728,12 @@
       </c>
       <c r="AD162" s="47" t="inlineStr">
         <is>
-          <t>B档，79分；字段显示主线为主线A-AI终端/智能硬件/TPM/软硬件协同项目，匹配度高，原申请优先级P2今日可投。城市/薪资为深圳/上海、Apple官网未公开，薪资匹配为实习薪资未公开；Apple平台价值高，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：全球消费电子与软硬件一体化顶级外企，AI终端、硬件工程、供应链和产品体验平台价值极高；JD与可信度为Apple官方搜索页可核验标题、发…、中高，扩源入口需后置核验。关键风险：薪资待确认；JD不精确；英文/粤语/IANG；招聘状态不稳。</t>
+          <t>B档，79分；字段显示主线为主线A-AI终端/智能硬件/TPM/软硬件协同项目，匹配度高，原申请优先级P2今日可投。城市/薪资为深圳/上海、Apple官网未公开，薪资匹配为实习薪资未公开；Apple平台价值高，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：全球消费电子与软硬件一体化顶级外企，AI终端、硬件工程、供应链和产品体验平台价值极高；JD与可信度为Apple官方搜索页可核验标题、发…、中高，入池岗位。关键风险：薪资待确认；JD不精确；英文/粤语/IANG；招聘状态不稳。</t>
         </is>
       </c>
       <c r="AE162" s="47" t="inlineStr">
         <is>
-          <t>作为主投池，持续监控</t>
+          <t>二次核验后投</t>
         </is>
       </c>
       <c r="AF162" s="47" t="inlineStr">
@@ -58197,7 +58197,7 @@
       </c>
       <c r="S7" s="47" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接无法精确确认（403），需二次确认；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
         </is>
       </c>
       <c r="T7" s="47" t="inlineStr">
@@ -58269,11 +58269,11 @@
         </is>
       </c>
       <c r="AH7" s="2" t="n">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="AI7" s="2" t="inlineStr">
         <is>
-          <t>B档，73分；字段显示主线为备线C-AI解决方案/数字化产品，匹配度中高，原申请优先级P2验证。城市/薪资为香港、未写，薪资匹配为待确认，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：香港本地ERP/企业系统厂商，正在把AI/CRM/ERP打包为企业数字化方案；JD与可信度为搜索结果核验、中，扩源入口需后置核验。关键风险：薪资待确认；英文/粤语/IANG；招聘状态不稳。</t>
+          <t>B档，76分；字段显示主线为备线C-AI解决方案/数字化产品，匹配度中高，原申请优先级P2验证。城市/薪资为香港、未写，薪资匹配为待确认，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：香港本地ERP/企业系统厂商，正在把AI/CRM/ERP打包为企业数字化方案；JD与可信度为搜索结果核验、中，扩源入口需后置核验。关键风险：薪资待确认；英文/粤语/IANG。</t>
         </is>
       </c>
       <c r="AJ7" s="2" t="inlineStr">
@@ -58283,7 +58283,7 @@
       </c>
       <c r="AK7" s="2" t="inlineStr">
         <is>
-          <t>薪资待确认；英文/粤语/IANG；招聘状态不稳</t>
+          <t>薪资待确认；英文/粤语/IANG</t>
         </is>
       </c>
       <c r="AL7" s="2" t="inlineStr">
@@ -58573,7 +58573,7 @@
       </c>
       <c r="S9" s="47" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接无法精确确认（403），需二次确认；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
         </is>
       </c>
       <c r="T9" s="47" t="inlineStr">
@@ -58745,7 +58745,7 @@
       </c>
       <c r="S10" s="47" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接无法精确确认（403），需二次确认；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
         </is>
       </c>
       <c r="T10" s="47" t="inlineStr">
@@ -59949,7 +59949,7 @@
       </c>
       <c r="S17" s="47" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接无法精确确认（429），需二次确认；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
         </is>
       </c>
       <c r="T17" s="47" t="inlineStr">
@@ -60009,17 +60009,17 @@
       </c>
       <c r="AI17" s="2" t="inlineStr">
         <is>
-          <t>C档，50分；字段显示主线为主线A-AIoT/AI终端/软硬件产品，匹配度高，原申请优先级P3次选验证。城市/薪资为香港、未写，薪资匹配为待确认，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：全球外设龙头与瑞士国际品牌；JD与可信度为精确JD、高，扩源入口需后置核验。关键风险：资深/高年限硬门槛：标题含高级/资深/专家/负责人/Lead/Owner等资深信号；详情或任职要求含5年及以上/5+ years硬经验门槛；薪资待确认；经验偏高；英文/粤语/IANG；出差/驻厂；招聘状态不稳。</t>
+          <t>C档，50分；字段显示主线为主线A-AIoT/AI终端/软硬件产品，匹配度高，原申请优先级P3次选验证。城市/薪资为香港、未写，薪资匹配为待确认，对当前香港/深圳双线与现金流目标的支撑不同。公司/岗位价值：全球外设龙头与瑞士国际品牌；JD与可信度为精确JD、高，扩源入口需后置核验。关键风险：资深/高年限硬门槛：标题含高级/资深/专家/负责人/Lead/Owner等资深信号；详情或任职要求含5年及以上/5+ years硬经验门槛；薪资待确认；经验偏高；英文/粤语/IANG；出差/驻厂。</t>
         </is>
       </c>
       <c r="AJ17" s="2" t="inlineStr">
         <is>
-          <t>观察</t>
+          <t>练手投/暂缓</t>
         </is>
       </c>
       <c r="AK17" s="2" t="inlineStr">
         <is>
-          <t>资深/高年限硬门槛：标题含高级/资深/专家/负责人/Lead/Owner等资深信号；详情或任职要求含5年及以上/5+ years硬经验门槛；薪资待确认；经验偏高；英文/粤语/IANG；出差/驻厂；招聘状态不稳</t>
+          <t>资深/高年限硬门槛：标题含高级/资深/专家/负责人/Lead/Owner等资深信号；详情或任职要求含5年及以上/5+ years硬经验门槛；薪资待确认；经验偏高；英文/粤语/IANG；出差/驻厂</t>
         </is>
       </c>
       <c r="AL17" s="2" t="inlineStr">
@@ -60873,7 +60873,7 @@
       </c>
       <c r="S22" s="47" t="inlineStr">
         <is>
-          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面内容较上次有变化；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
+          <t>2026-06-17 自动复核：链接可打开，未识别下架关键词；页面未公开HR活跃/登录状态；不绕过登录或反爬抓取</t>
         </is>
       </c>
       <c r="T22" s="47" t="inlineStr">
@@ -61595,7 +61595,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E211"/>
+  <dimension ref="A1:E228"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -64961,6 +64961,261 @@
       <c r="C211" s="48" t="n"/>
       <c r="D211" s="48" t="n"/>
       <c r="E211" s="48" t="n"/>
+    </row>
+    <row r="212">
+      <c r="A212" s="48" t="inlineStr">
+        <is>
+          <t>新明珠集团</t>
+        </is>
+      </c>
+      <c r="B212" s="48" t="inlineStr">
+        <is>
+          <t>AI智能体产品设计师</t>
+        </is>
+      </c>
+      <c r="C212" s="48" t="inlineStr"/>
+      <c r="D212" s="48" t="inlineStr"/>
+      <c r="E212" s="48" t="inlineStr"/>
+    </row>
+    <row r="213">
+      <c r="A213" s="48" t="inlineStr">
+        <is>
+          <t>玖龙纸业（控股）有限公司</t>
+        </is>
+      </c>
+      <c r="B213" s="48" t="inlineStr">
+        <is>
+          <t>AI产品经理</t>
+        </is>
+      </c>
+      <c r="C213" s="48" t="inlineStr"/>
+      <c r="D213" s="48" t="inlineStr"/>
+      <c r="E213" s="48" t="inlineStr"/>
+    </row>
+    <row r="214">
+      <c r="A214" s="48" t="inlineStr">
+        <is>
+          <t>Seeed 矽递科技</t>
+        </is>
+      </c>
+      <c r="B214" s="48" t="inlineStr">
+        <is>
+          <t>AI产品经理</t>
+        </is>
+      </c>
+      <c r="C214" s="48" t="inlineStr"/>
+      <c r="D214" s="48" t="inlineStr"/>
+      <c r="E214" s="48" t="inlineStr"/>
+    </row>
+    <row r="215">
+      <c r="A215" s="48" t="inlineStr">
+        <is>
+          <t>深圳欣盛商科技有限公司</t>
+        </is>
+      </c>
+      <c r="B215" s="48" t="inlineStr">
+        <is>
+          <t>企业AI应用工程师</t>
+        </is>
+      </c>
+      <c r="C215" s="48" t="inlineStr"/>
+      <c r="D215" s="48" t="inlineStr"/>
+      <c r="E215" s="48" t="inlineStr"/>
+    </row>
+    <row r="216">
+      <c r="A216" s="48" t="inlineStr">
+        <is>
+          <t>美团</t>
+        </is>
+      </c>
+      <c r="B216" s="48" t="inlineStr">
+        <is>
+          <t>AI硬件产品专员/工程师</t>
+        </is>
+      </c>
+      <c r="C216" s="48" t="inlineStr"/>
+      <c r="D216" s="48" t="inlineStr"/>
+      <c r="E216" s="48" t="inlineStr"/>
+    </row>
+    <row r="217">
+      <c r="A217" s="48" t="inlineStr">
+        <is>
+          <t>深圳启奥人工智能科技有限公司</t>
+        </is>
+      </c>
+      <c r="B217" s="48" t="inlineStr">
+        <is>
+          <t>产品经理</t>
+        </is>
+      </c>
+      <c r="C217" s="48" t="inlineStr"/>
+      <c r="D217" s="48" t="inlineStr"/>
+      <c r="E217" s="48" t="inlineStr"/>
+    </row>
+    <row r="218">
+      <c r="A218" s="48" t="inlineStr">
+        <is>
+          <t>深圳费曼智核机器人科技有限公司</t>
+        </is>
+      </c>
+      <c r="B218" s="48" t="inlineStr">
+        <is>
+          <t>大模型产品经理</t>
+        </is>
+      </c>
+      <c r="C218" s="48" t="inlineStr"/>
+      <c r="D218" s="48" t="inlineStr"/>
+      <c r="E218" s="48" t="inlineStr"/>
+    </row>
+    <row r="219">
+      <c r="A219" s="48" t="inlineStr">
+        <is>
+          <t>鱼泡直聘线索/深圳宝安未核验雇主</t>
+        </is>
+      </c>
+      <c r="B219" s="48" t="inlineStr">
+        <is>
+          <t>工业AI产品经理</t>
+        </is>
+      </c>
+      <c r="C219" s="48" t="inlineStr"/>
+      <c r="D219" s="48" t="inlineStr"/>
+      <c r="E219" s="48" t="inlineStr"/>
+    </row>
+    <row r="220">
+      <c r="A220" s="48" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="B220" s="48" t="inlineStr">
+        <is>
+          <t>Subject Matter Expert - Automation &amp; AI/ML</t>
+        </is>
+      </c>
+      <c r="C220" s="48" t="inlineStr"/>
+      <c r="D220" s="48" t="inlineStr"/>
+      <c r="E220" s="48" t="inlineStr"/>
+    </row>
+    <row r="221">
+      <c r="A221" s="48" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="B221" s="48" t="inlineStr">
+        <is>
+          <t>Machine Learning &amp; AI Engineer</t>
+        </is>
+      </c>
+      <c r="C221" s="48" t="inlineStr"/>
+      <c r="D221" s="48" t="inlineStr"/>
+      <c r="E221" s="48" t="inlineStr"/>
+    </row>
+    <row r="222">
+      <c r="A222" s="48" t="inlineStr">
+        <is>
+          <t>Reap</t>
+        </is>
+      </c>
+      <c r="B222" s="48" t="inlineStr">
+        <is>
+          <t>Technical Product Manager, AI Platform</t>
+        </is>
+      </c>
+      <c r="C222" s="48" t="inlineStr"/>
+      <c r="D222" s="48" t="inlineStr"/>
+      <c r="E222" s="48" t="inlineStr"/>
+    </row>
+    <row r="223">
+      <c r="A223" s="48" t="inlineStr">
+        <is>
+          <t>深圳中博纳网络科技有限公司（鱼泡直聘线索）</t>
+        </is>
+      </c>
+      <c r="B223" s="48" t="inlineStr">
+        <is>
+          <t>AI+机器人产品经理</t>
+        </is>
+      </c>
+      <c r="C223" s="48" t="inlineStr"/>
+      <c r="D223" s="48" t="inlineStr"/>
+      <c r="E223" s="48" t="inlineStr"/>
+    </row>
+    <row r="224">
+      <c r="A224" s="48" t="inlineStr">
+        <is>
+          <t>科大讯飞硬件中心</t>
+        </is>
+      </c>
+      <c r="B224" s="48" t="inlineStr">
+        <is>
+          <t>高级平台硬件产品经理（机器人）</t>
+        </is>
+      </c>
+      <c r="C224" s="48" t="inlineStr"/>
+      <c r="D224" s="48" t="inlineStr"/>
+      <c r="E224" s="48" t="inlineStr"/>
+    </row>
+    <row r="225">
+      <c r="A225" s="48" t="inlineStr">
+        <is>
+          <t>中电信数智科技(深圳)有限公司</t>
+        </is>
+      </c>
+      <c r="B225" s="48" t="inlineStr">
+        <is>
+          <t>智能组网产品经理</t>
+        </is>
+      </c>
+      <c r="C225" s="48" t="inlineStr"/>
+      <c r="D225" s="48" t="inlineStr"/>
+      <c r="E225" s="48" t="inlineStr"/>
+    </row>
+    <row r="226">
+      <c r="A226" s="48" t="inlineStr">
+        <is>
+          <t>New Media Group Publishing Limited</t>
+        </is>
+      </c>
+      <c r="B226" s="48" t="inlineStr">
+        <is>
+          <t>Product Manager - AI Rich Media Solution</t>
+        </is>
+      </c>
+      <c r="C226" s="48" t="inlineStr"/>
+      <c r="D226" s="48" t="inlineStr"/>
+      <c r="E226" s="48" t="inlineStr"/>
+    </row>
+    <row r="227">
+      <c r="A227" s="48" t="inlineStr">
+        <is>
+          <t>Galaxy Telecom (Hong Kong) Limited</t>
+        </is>
+      </c>
+      <c r="B227" s="48" t="inlineStr">
+        <is>
+          <t>AI Product Manager / Owner (ERP project)</t>
+        </is>
+      </c>
+      <c r="C227" s="48" t="inlineStr"/>
+      <c r="D227" s="48" t="inlineStr"/>
+      <c r="E227" s="48" t="inlineStr"/>
+    </row>
+    <row r="228">
+      <c r="A228" s="48" t="inlineStr">
+        <is>
+          <t>HK01 Company Limited</t>
+        </is>
+      </c>
+      <c r="B228" s="48" t="inlineStr">
+        <is>
+          <t>AI Application Product Manager</t>
+        </is>
+      </c>
+      <c r="C228" s="48" t="inlineStr"/>
+      <c r="D228" s="48" t="inlineStr"/>
+      <c r="E228" s="48" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:E16"/>

</xml_diff>